<commit_message>
update report for 2024 data
</commit_message>
<xml_diff>
--- a/effortbbdataGreatRiverGreening.xlsx
+++ b/effortbbdataGreatRiverGreening.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\R\greatrivergreeningbumblebees\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{042FD892-8F0B-4D2A-9595-D3312BB40B55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3730E1E0-027E-468C-9F38-BA05F9F81E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15705" yWindow="0" windowWidth="18225" windowHeight="14760"/>
+    <workbookView xWindow="1290" yWindow="-110" windowWidth="18020" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="effortbbdataGreatRiverGreening" sheetId="1" r:id="rId1"/>
@@ -589,7 +589,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1425,16 +1425,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U274"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" customWidth="1"/>
-    <col min="9" max="9" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.54296875" customWidth="1"/>
+    <col min="9" max="9" width="13.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>129</v>
       </c>
@@ -1499,7 +1499,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1564,7 +1564,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1629,7 +1629,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1694,7 +1694,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1759,7 +1759,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1824,7 +1824,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1889,7 +1889,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1954,7 +1954,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2019,7 +2019,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2084,7 +2084,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2149,7 +2149,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2214,7 +2214,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2279,7 +2279,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2344,7 +2344,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2409,7 +2409,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2474,7 +2474,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2539,7 +2539,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2604,7 +2604,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2669,7 +2669,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2734,7 +2734,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2799,7 +2799,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2864,7 +2864,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2929,7 +2929,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2994,7 +2994,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>24</v>
       </c>
@@ -3059,7 +3059,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>25</v>
       </c>
@@ -3124,7 +3124,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>26</v>
       </c>
@@ -3189,7 +3189,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>27</v>
       </c>
@@ -3254,7 +3254,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>28</v>
       </c>
@@ -3319,7 +3319,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>29</v>
       </c>
@@ -3378,7 +3378,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>30</v>
       </c>
@@ -3437,7 +3437,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>31</v>
       </c>
@@ -3502,7 +3502,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>32</v>
       </c>
@@ -3567,7 +3567,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>33</v>
       </c>
@@ -3632,7 +3632,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>34</v>
       </c>
@@ -3697,7 +3697,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>35</v>
       </c>
@@ -3762,7 +3762,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>36</v>
       </c>
@@ -3827,7 +3827,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>37</v>
       </c>
@@ -3892,7 +3892,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>38</v>
       </c>
@@ -3957,7 +3957,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>39</v>
       </c>
@@ -4022,7 +4022,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>40</v>
       </c>
@@ -4087,7 +4087,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>41</v>
       </c>
@@ -4152,7 +4152,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>42</v>
       </c>
@@ -4217,7 +4217,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>43</v>
       </c>
@@ -4282,7 +4282,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>44</v>
       </c>
@@ -4347,7 +4347,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>45</v>
       </c>
@@ -4412,7 +4412,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>46</v>
       </c>
@@ -4477,7 +4477,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>47</v>
       </c>
@@ -4542,7 +4542,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="49" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>48</v>
       </c>
@@ -4607,7 +4607,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="50" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>49</v>
       </c>
@@ -4672,7 +4672,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="51" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>50</v>
       </c>
@@ -4737,7 +4737,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="52" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>51</v>
       </c>
@@ -4802,7 +4802,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>52</v>
       </c>
@@ -4867,7 +4867,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>53</v>
       </c>
@@ -4932,7 +4932,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="55" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>54</v>
       </c>
@@ -4997,7 +4997,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="56" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>55</v>
       </c>
@@ -5056,7 +5056,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="57" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>56</v>
       </c>
@@ -5121,7 +5121,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="58" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>57</v>
       </c>
@@ -5180,7 +5180,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="59" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>58</v>
       </c>
@@ -5239,7 +5239,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="60" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>59</v>
       </c>
@@ -5298,7 +5298,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="61" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>60</v>
       </c>
@@ -5357,7 +5357,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="62" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>61</v>
       </c>
@@ -5416,7 +5416,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="63" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>62</v>
       </c>
@@ -5475,7 +5475,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="64" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>63</v>
       </c>
@@ -5534,7 +5534,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>64</v>
       </c>
@@ -5593,7 +5593,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>65</v>
       </c>
@@ -5652,7 +5652,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>66</v>
       </c>
@@ -5711,7 +5711,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>67</v>
       </c>
@@ -5770,7 +5770,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>68</v>
       </c>
@@ -5829,7 +5829,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>69</v>
       </c>
@@ -5888,7 +5888,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>70</v>
       </c>
@@ -5947,7 +5947,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>71</v>
       </c>
@@ -6006,7 +6006,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="73" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>72</v>
       </c>
@@ -6065,7 +6065,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="74" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>73</v>
       </c>
@@ -6124,7 +6124,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="75" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>74</v>
       </c>
@@ -6183,7 +6183,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="76" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>75</v>
       </c>
@@ -6242,7 +6242,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="77" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>76</v>
       </c>
@@ -6301,7 +6301,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="78" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>77</v>
       </c>
@@ -6360,7 +6360,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="79" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>78</v>
       </c>
@@ -6419,7 +6419,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="80" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>79</v>
       </c>
@@ -6478,7 +6478,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>80</v>
       </c>
@@ -6537,7 +6537,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>81</v>
       </c>
@@ -6596,7 +6596,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="83" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>82</v>
       </c>
@@ -6655,7 +6655,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>83</v>
       </c>
@@ -6714,7 +6714,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>84</v>
       </c>
@@ -6773,7 +6773,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>85</v>
       </c>
@@ -6832,7 +6832,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>86</v>
       </c>
@@ -6891,7 +6891,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>87</v>
       </c>
@@ -6950,7 +6950,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="89" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>88</v>
       </c>
@@ -7009,7 +7009,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="90" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>89</v>
       </c>
@@ -7068,7 +7068,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="91" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A91">
         <v>90</v>
       </c>
@@ -7127,7 +7127,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="92" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>91</v>
       </c>
@@ -7186,7 +7186,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="93" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>92</v>
       </c>
@@ -7245,7 +7245,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="94" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>93</v>
       </c>
@@ -7304,7 +7304,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="95" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A95">
         <v>94</v>
       </c>
@@ -7363,7 +7363,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="96" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>95</v>
       </c>
@@ -7422,7 +7422,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>96</v>
       </c>
@@ -7481,7 +7481,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>97</v>
       </c>
@@ -7540,7 +7540,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="99" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>98</v>
       </c>
@@ -7602,7 +7602,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="100" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>99</v>
       </c>
@@ -7664,7 +7664,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="101" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A101">
         <v>100</v>
       </c>
@@ -7726,7 +7726,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="102" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A102">
         <v>101</v>
       </c>
@@ -7788,7 +7788,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="103" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>102</v>
       </c>
@@ -7850,7 +7850,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="104" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>103</v>
       </c>
@@ -7912,7 +7912,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="105" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A105">
         <v>104</v>
       </c>
@@ -7974,7 +7974,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="106" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A106">
         <v>105</v>
       </c>
@@ -8036,7 +8036,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="107" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A107">
         <v>106</v>
       </c>
@@ -8098,7 +8098,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="108" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A108">
         <v>107</v>
       </c>
@@ -8160,7 +8160,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="109" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A109">
         <v>108</v>
       </c>
@@ -8222,7 +8222,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="110" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A110">
         <v>109</v>
       </c>
@@ -8281,7 +8281,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="111" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A111">
         <v>110</v>
       </c>
@@ -8340,7 +8340,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="112" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A112">
         <v>111</v>
       </c>
@@ -8399,7 +8399,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="113" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A113">
         <v>112</v>
       </c>
@@ -8458,7 +8458,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="114" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A114">
         <v>113</v>
       </c>
@@ -8520,7 +8520,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="115" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A115">
         <v>114</v>
       </c>
@@ -8579,7 +8579,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="116" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A116">
         <v>115</v>
       </c>
@@ -8638,7 +8638,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="117" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>116</v>
       </c>
@@ -8697,7 +8697,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="118" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>117</v>
       </c>
@@ -8762,7 +8762,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="119" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>118</v>
       </c>
@@ -8824,7 +8824,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="120" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>119</v>
       </c>
@@ -8883,7 +8883,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="121" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A121">
         <v>120</v>
       </c>
@@ -8942,7 +8942,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="122" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>121</v>
       </c>
@@ -9001,7 +9001,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="123" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A123">
         <v>122</v>
       </c>
@@ -9060,7 +9060,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="124" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A124">
         <v>123</v>
       </c>
@@ -9119,7 +9119,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="125" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A125">
         <v>124</v>
       </c>
@@ -9178,7 +9178,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="126" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A126">
         <v>125</v>
       </c>
@@ -9240,7 +9240,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="127" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A127">
         <v>126</v>
       </c>
@@ -9299,7 +9299,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="128" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A128">
         <v>127</v>
       </c>
@@ -9358,7 +9358,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="129" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A129">
         <v>128</v>
       </c>
@@ -9417,7 +9417,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="130" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A130">
         <v>129</v>
       </c>
@@ -9476,7 +9476,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="131" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A131">
         <v>130</v>
       </c>
@@ -9535,7 +9535,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="132" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A132">
         <v>131</v>
       </c>
@@ -9597,7 +9597,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="133" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A133">
         <v>132</v>
       </c>
@@ -9659,7 +9659,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="134" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A134">
         <v>133</v>
       </c>
@@ -9721,7 +9721,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="135" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A135">
         <v>134</v>
       </c>
@@ -9780,7 +9780,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="136" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A136">
         <v>135</v>
       </c>
@@ -9839,7 +9839,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="137" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A137">
         <v>136</v>
       </c>
@@ -9898,7 +9898,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="138" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A138">
         <v>137</v>
       </c>
@@ -9957,7 +9957,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="139" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A139">
         <v>138</v>
       </c>
@@ -10016,7 +10016,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="140" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A140">
         <v>139</v>
       </c>
@@ -10075,7 +10075,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="141" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A141">
         <v>140</v>
       </c>
@@ -10134,7 +10134,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="142" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A142">
         <v>141</v>
       </c>
@@ -10193,7 +10193,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="143" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A143">
         <v>142</v>
       </c>
@@ -10252,7 +10252,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="144" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A144">
         <v>143</v>
       </c>
@@ -10311,7 +10311,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="145" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A145">
         <v>144</v>
       </c>
@@ -10373,7 +10373,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="146" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A146">
         <v>145</v>
       </c>
@@ -10432,7 +10432,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="147" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A147">
         <v>146</v>
       </c>
@@ -10491,7 +10491,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="148" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A148">
         <v>147</v>
       </c>
@@ -10550,7 +10550,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="149" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A149">
         <v>148</v>
       </c>
@@ -10612,7 +10612,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="150" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A150">
         <v>149</v>
       </c>
@@ -10671,7 +10671,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="151" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A151">
         <v>150</v>
       </c>
@@ -10730,7 +10730,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="152" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A152">
         <v>151</v>
       </c>
@@ -10789,7 +10789,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="153" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A153">
         <v>152</v>
       </c>
@@ -10848,7 +10848,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="154" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A154">
         <v>153</v>
       </c>
@@ -10910,7 +10910,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="155" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A155">
         <v>154</v>
       </c>
@@ -10972,7 +10972,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="156" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A156">
         <v>155</v>
       </c>
@@ -11034,7 +11034,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="157" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A157">
         <v>156</v>
       </c>
@@ -11096,7 +11096,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="158" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A158">
         <v>157</v>
       </c>
@@ -11158,7 +11158,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="159" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A159">
         <v>158</v>
       </c>
@@ -11220,7 +11220,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="160" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A160">
         <v>159</v>
       </c>
@@ -11282,7 +11282,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="161" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A161">
         <v>160</v>
       </c>
@@ -11341,7 +11341,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="162" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A162">
         <v>161</v>
       </c>
@@ -11400,7 +11400,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="163" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A163">
         <v>162</v>
       </c>
@@ -11459,7 +11459,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="164" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A164">
         <v>163</v>
       </c>
@@ -11518,7 +11518,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="165" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A165">
         <v>164</v>
       </c>
@@ -11577,7 +11577,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="166" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A166">
         <v>165</v>
       </c>
@@ -11636,7 +11636,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="167" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A167">
         <v>166</v>
       </c>
@@ -11695,7 +11695,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="168" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A168">
         <v>167</v>
       </c>
@@ -11754,7 +11754,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="169" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A169">
         <v>168</v>
       </c>
@@ -11813,7 +11813,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="170" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A170">
         <v>169</v>
       </c>
@@ -11872,7 +11872,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="171" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A171">
         <v>170</v>
       </c>
@@ -11931,7 +11931,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="172" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A172">
         <v>171</v>
       </c>
@@ -11990,7 +11990,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="173" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A173">
         <v>172</v>
       </c>
@@ -12049,7 +12049,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="174" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A174">
         <v>173</v>
       </c>
@@ -12108,7 +12108,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="175" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A175">
         <v>174</v>
       </c>
@@ -12167,7 +12167,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="176" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A176">
         <v>175</v>
       </c>
@@ -12226,7 +12226,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="177" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A177">
         <v>176</v>
       </c>
@@ -12285,7 +12285,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="178" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A178">
         <v>177</v>
       </c>
@@ -12344,7 +12344,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="179" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A179">
         <v>178</v>
       </c>
@@ -12403,7 +12403,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="180" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A180">
         <v>179</v>
       </c>
@@ -12462,7 +12462,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="181" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A181">
         <v>180</v>
       </c>
@@ -12521,7 +12521,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="182" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A182">
         <v>181</v>
       </c>
@@ -12580,7 +12580,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="183" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A183">
         <v>182</v>
       </c>
@@ -12639,7 +12639,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="184" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A184">
         <v>183</v>
       </c>
@@ -12698,7 +12698,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="185" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A185">
         <v>184</v>
       </c>
@@ -12757,7 +12757,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="186" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A186">
         <v>185</v>
       </c>
@@ -12816,7 +12816,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="187" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A187">
         <v>186</v>
       </c>
@@ -12875,7 +12875,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="188" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A188">
         <v>187</v>
       </c>
@@ -12934,7 +12934,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="189" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A189">
         <v>188</v>
       </c>
@@ -12993,7 +12993,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="190" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A190">
         <v>189</v>
       </c>
@@ -13052,7 +13052,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="191" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A191">
         <v>190</v>
       </c>
@@ -13111,7 +13111,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="192" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A192">
         <v>191</v>
       </c>
@@ -13170,7 +13170,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="193" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A193">
         <v>192</v>
       </c>
@@ -13229,7 +13229,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="194" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A194">
         <v>193</v>
       </c>
@@ -13288,7 +13288,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="195" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A195">
         <v>194</v>
       </c>
@@ -13347,7 +13347,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="196" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A196">
         <v>195</v>
       </c>
@@ -13406,7 +13406,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="197" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A197">
         <v>196</v>
       </c>
@@ -13465,7 +13465,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="198" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A198">
         <v>197</v>
       </c>
@@ -13521,7 +13521,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="199" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A199">
         <v>198</v>
       </c>
@@ -13580,7 +13580,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="200" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A200">
         <v>199</v>
       </c>
@@ -13639,7 +13639,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="201" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A201">
         <v>200</v>
       </c>
@@ -13698,7 +13698,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="202" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A202">
         <v>201</v>
       </c>
@@ -13757,7 +13757,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="203" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A203">
         <v>202</v>
       </c>
@@ -13816,7 +13816,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="204" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A204">
         <v>203</v>
       </c>
@@ -13872,7 +13872,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="205" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A205">
         <v>204</v>
       </c>
@@ -13931,7 +13931,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="206" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A206">
         <v>205</v>
       </c>
@@ -13990,7 +13990,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="207" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A207">
         <v>206</v>
       </c>
@@ -14049,7 +14049,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="208" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A208">
         <v>207</v>
       </c>
@@ -14108,7 +14108,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="209" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A209">
         <v>208</v>
       </c>
@@ -14167,7 +14167,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="210" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A210">
         <v>209</v>
       </c>
@@ -14226,7 +14226,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="211" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A211">
         <v>210</v>
       </c>
@@ -14285,7 +14285,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="212" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A212">
         <v>211</v>
       </c>
@@ -14344,7 +14344,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="213" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A213">
         <v>212</v>
       </c>
@@ -14403,7 +14403,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="214" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A214">
         <v>213</v>
       </c>
@@ -14462,7 +14462,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="215" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A215">
         <v>214</v>
       </c>
@@ -14524,7 +14524,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="216" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A216">
         <v>215</v>
       </c>
@@ -14583,7 +14583,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="217" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A217">
         <v>216</v>
       </c>
@@ -14645,7 +14645,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="218" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A218">
         <v>217</v>
       </c>
@@ -14707,7 +14707,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="219" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A219">
         <v>218</v>
       </c>
@@ -14769,7 +14769,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="220" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A220">
         <v>219</v>
       </c>
@@ -14828,7 +14828,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="221" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A221">
         <v>220</v>
       </c>
@@ -14887,7 +14887,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="222" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A222">
         <v>221</v>
       </c>
@@ -14946,7 +14946,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="223" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A223">
         <v>222</v>
       </c>
@@ -15002,7 +15002,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="224" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A224">
         <v>223</v>
       </c>
@@ -15061,7 +15061,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="225" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A225">
         <v>224</v>
       </c>
@@ -15120,7 +15120,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="226" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A226">
         <v>225</v>
       </c>
@@ -15179,7 +15179,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="227" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A227">
         <v>226</v>
       </c>
@@ -15238,7 +15238,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="228" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A228">
         <v>227</v>
       </c>
@@ -15297,7 +15297,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="229" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A229">
         <v>228</v>
       </c>
@@ -15356,7 +15356,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="230" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A230">
         <v>229</v>
       </c>
@@ -15415,7 +15415,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="231" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A231">
         <v>230</v>
       </c>
@@ -15474,7 +15474,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="232" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A232">
         <v>231</v>
       </c>
@@ -15533,7 +15533,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="233" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A233">
         <v>232</v>
       </c>
@@ -15592,7 +15592,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="234" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A234">
         <v>233</v>
       </c>
@@ -15651,7 +15651,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="235" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A235">
         <v>234</v>
       </c>
@@ -15710,7 +15710,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="236" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A236">
         <v>235</v>
       </c>
@@ -15769,7 +15769,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="237" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A237">
         <v>236</v>
       </c>
@@ -15828,7 +15828,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="238" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A238">
         <v>237</v>
       </c>
@@ -15887,7 +15887,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="239" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A239">
         <v>238</v>
       </c>
@@ -15946,7 +15946,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="240" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A240">
         <v>239</v>
       </c>
@@ -16002,7 +16002,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="241" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A241">
         <v>240</v>
       </c>
@@ -16061,7 +16061,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="242" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A242">
         <v>241</v>
       </c>
@@ -16120,7 +16120,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="243" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A243">
         <v>242</v>
       </c>
@@ -16179,7 +16179,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="244" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A244">
         <v>243</v>
       </c>
@@ -16238,7 +16238,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="245" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A245">
         <v>244</v>
       </c>
@@ -16297,7 +16297,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="246" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A246">
         <v>245</v>
       </c>
@@ -16356,7 +16356,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="247" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A247">
         <v>246</v>
       </c>
@@ -16415,7 +16415,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="248" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A248">
         <v>247</v>
       </c>
@@ -16474,7 +16474,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="249" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A249">
         <v>248</v>
       </c>
@@ -16533,7 +16533,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="250" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A250">
         <v>249</v>
       </c>
@@ -16592,7 +16592,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="251" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A251">
         <v>250</v>
       </c>
@@ -16651,7 +16651,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="252" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A252">
         <v>251</v>
       </c>
@@ -16710,7 +16710,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="253" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A253">
         <v>252</v>
       </c>
@@ -16769,7 +16769,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="254" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A254">
         <v>253</v>
       </c>
@@ -16825,7 +16825,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="255" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A255">
         <v>254</v>
       </c>
@@ -16884,7 +16884,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="256" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A256">
         <v>255</v>
       </c>
@@ -16943,7 +16943,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="257" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A257">
         <v>256</v>
       </c>
@@ -17002,7 +17002,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="258" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A258">
         <v>257</v>
       </c>
@@ -17061,7 +17061,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="259" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A259">
         <v>258</v>
       </c>
@@ -17120,7 +17120,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="260" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A260">
         <v>259</v>
       </c>
@@ -17179,7 +17179,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="261" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A261">
         <v>260</v>
       </c>
@@ -17238,7 +17238,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="262" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A262">
         <v>261</v>
       </c>
@@ -17294,7 +17294,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="263" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A263">
         <v>262</v>
       </c>
@@ -17353,7 +17353,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="264" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A264">
         <v>263</v>
       </c>
@@ -17412,7 +17412,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="265" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A265">
         <v>264</v>
       </c>
@@ -17471,7 +17471,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="266" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A266">
         <v>265</v>
       </c>
@@ -17530,7 +17530,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="267" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A267">
         <v>266</v>
       </c>
@@ -17589,7 +17589,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="268" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A268">
         <v>267</v>
       </c>
@@ -17648,7 +17648,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="269" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A269">
         <v>268</v>
       </c>
@@ -17707,7 +17707,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="270" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A270">
         <v>269</v>
       </c>
@@ -17766,7 +17766,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="271" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A271">
         <v>270</v>
       </c>
@@ -17825,7 +17825,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="272" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A272">
         <v>271</v>
       </c>
@@ -17884,7 +17884,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="273" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A273">
         <v>272</v>
       </c>
@@ -17943,7 +17943,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="274" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A274">
         <v>273</v>
       </c>

</xml_diff>